<commit_message>
v1.38: Detalle clic en importe abre movimientos
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E98"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2008,16 +2008,84 @@
         <v>Fix</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B95" t="str">
+        <v>17:25</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Despliegue v1.37</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Fix scroll To-Do en celular vertical; everfit-release.json v1.37. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B96" t="str">
+        <v>17:26</v>
+      </c>
+      <c r="C96" t="str">
+        <v>To-Do: vaciar tablas para uso real</v>
+      </c>
+      <c r="D96" t="str">
+        <v>TRUNCATE de todo_instancia y todo_tarea (6 plantillas y 433 ocurrencias de prueba) para arrancar el menú To-Do en producción sin datos de prueba.</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Datos</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B97" t="str">
+        <v>10:46</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Detalle: clic en importe → movimientos</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Modal Detalle (solapas Concepto y Beneficiario): cada importe (mes o Total; ítem, fila Ingresos/Egresos o G/P) abre el modal Movimientos con las filas de base_everfit que suman ese valor (mismo filtro de sucursal, moneda/TC y exclusión Saldo Inicial; G/P con egresos en negativo). Tabla con thead sticky y total al pie, responsive, export Excel con importe numérico. Carga base_everfit suma detalle, medio y observaciones.</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B98" t="str">
+        <v>10:58</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Despliegue v1.38</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Drill-down de importes a movimientos en modal Detalle (ambas solapas) con export Excel; everfit-release.json v1.38. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E98"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -2105,23 +2173,31 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Sedes – catálogo ABM</v>
+        <v>Detalle por Concepto / Beneficiario – movimientos</v>
       </c>
       <c r="B11" t="str">
-        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+        <v>En el modal Detalle (clic en fila del Flujo por mes), cualquier importe de ambas solapas abre el listado de movimientos que lo componen: fecha de pago, tipo, concepto, beneficiario, centro de costos, detalle, medio, sucursal, real/pendiente, observaciones e importe, con total al pie y export Excel. Respeta sucursal, moneda ARS/USD y exclusión Saldo Inicial. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>Sedes – catálogo ABM</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>Configuración – reasignar To-Do</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B13" t="str">
         <v>Menú Configuración (permiso ver_configuracion, default Admin/Encargado). Reasignar una, varias o todas las tareas abiertas de un usuario a otro, o de un perfil a otro (p. ej. Recepcionista → Profesor). SQL: sql/supabase_todo_reasignar.sql. Docs: docs/CONFIGURACION.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2191,7 +2267,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C40"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2616,9 +2692,31 @@
         <v>To-Do: Mi perfil (nombre para mostrar); columna Usuario; tooltip email copiar en Responsable/Usuario; bandeja mobile (Acción 4.ª, scroll horizontal); modales nueva/editar responsive; permiso ver_dashboard; Seguridad edita nombre por usuario. SQL migraciones Supabase. everfit-release.json v1.36.</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>1.37</v>
+      </c>
+      <c r="B39" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="C39" t="str">
+        <v>To-Do: fix scroll bandeja en celular vertical (sin sticky Acción ≤768px, hint deslizar). everfit-release.json v1.37.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>1.38</v>
+      </c>
+      <c r="B40" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Modal Detalle (Concepto y Beneficiario): clic en cualquier importe abre modal Movimientos con las filas que lo componen (sucursal, moneda/TC, exclusión Saldo Inicial; G/P con egresos negativos), total al pie y export Excel. Carga base_everfit suma detalle, medio y observaciones. everfit-release.json v1.38.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.39: filtro Período, tendencia G/P y reporte PDF
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E102"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2076,16 +2076,84 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B99" t="str">
+        <v>11:28</v>
+      </c>
+      <c r="C99" t="str">
+        <v>G/P Mensual: tendencia y variación</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Gráfico G/P Mensual: línea de tendencia (mínimos cuadrados sobre 13 meses, punteada azul, en leyenda); variación vs mes anterior en monto y % sobre cada barra (con halo blanco; ocultas &lt;560 px) y en el tooltip; resumen «último mes vs anterior» y «Tendencia ±$ por mes». % sobre |mes anterior|; el primer mes compara con el previo no graficado. Ayuda (?) actualizada.</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B100" t="str">
+        <v>11:40</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Dashboard: reporte PDF con filtros activos</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Botón PDF (como Saldos extractos de Fornitalia): bloque de impresión A4 apaisado con encabezado (logo, fecha/hora AR, usuario, última actualización), recuadro de filtros con chips resaltados «Filtro activo» (sucursal / permisos, moneda USD y conversión) y parámetros informativos; tarjetas, gráfico G/P como imagen y tabla Flujo + ratios acotada a los 13 meses del gráfico + Proy. (Total recalculado), partida en bloques de columnas; notas. window.print y limpieza en afterprint. Barra: solo se oculta Actualizar base sin upload_base (antes se ocultaba todo el bloque derecho).</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B101" t="str">
+        <v>11:47</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Dashboard: filtro Período + PDF en miles</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Filtro Período después de Moneda (default Último año = mes actual AR + 12 anteriores, como el gráfico; años con datos; Todo el histórico), resaltado mientras recorta. Aplica a tarjetas, gráfico, tabla Flujo, ratios, Detalle, Movimientos y PDF. Proy. solo si el período incluye el mes en curso, con base en historia completa. Reporte PDF: importes en miles (aviso, encabezado y notas), sin meses proyectados, tabla en una hoja con 13 meses + Total.</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Feature</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B102" t="str">
+        <v>11:49</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Despliegue v1.39</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Filtro Período, tendencia y variación en G/P Mensual, reporte PDF con filtros resaltados e importes en miles; everfit-release.json v1.39. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E102"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B16"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -2173,31 +2241,55 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Detalle por Concepto / Beneficiario – movimientos</v>
+        <v>Gráfico G/P Mensual – tendencia y variación</v>
       </c>
       <c r="B11" t="str">
-        <v>En el modal Detalle (clic en fila del Flujo por mes), cualquier importe de ambas solapas abre el listado de movimientos que lo componen: fecha de pago, tipo, concepto, beneficiario, centro de costos, detalle, medio, sucursal, real/pendiente, observaciones e importe, con total al pie y export Excel. Respeta sucursal, moneda ARS/USD y exclusión Saldo Inicial. Docs: docs/DASHBOARD.md.</v>
+        <v>Barras G/P de 13 meses con línea de tendencia lineal y variación vs mes anterior (monto abreviado y %) sobre cada barra y en tooltip; resumen del último mes vs anterior y pendiente de la tendencia por mes. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Sedes – catálogo ABM</v>
+        <v>Dashboard – filtro Período</v>
       </c>
       <c r="B12" t="str">
-        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+        <v>Selector Período (Último año por defecto, años, Todo el histórico) que filtra por mes de fecha_pago tarjetas, gráfico G/P, Flujo por mes, ratios, Detalle, Movimientos y PDF. Proyección solo si el período incluye el mes en curso. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>Dashboard – reporte PDF</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Botón PDF en la barra de filtros: reporte imprimible (Guardar como PDF) con filtros activos resaltados, importes en miles, tarjetas, gráfico G/P y tabla Flujo por mes + ratios del período elegido, sin meses proyectados. Docs: docs/DASHBOARD.md.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Detalle por Concepto / Beneficiario – movimientos</v>
+      </c>
+      <c r="B14" t="str">
+        <v>En el modal Detalle (clic en fila del Flujo por mes), cualquier importe de ambas solapas abre el listado de movimientos que lo componen: fecha de pago, tipo, concepto, beneficiario, centro de costos, detalle, medio, sucursal, real/pendiente, observaciones e importe, con total al pie y export Excel. Respeta sucursal, moneda ARS/USD y exclusión Saldo Inicial. Docs: docs/DASHBOARD.md.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Sedes – catálogo ABM</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>Configuración – reasignar To-Do</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B16" t="str">
         <v>Menú Configuración (permiso ver_configuracion, default Admin/Encargado). Reasignar una, varias o todas las tareas abiertas de un usuario a otro, o de un perfil a otro (p. ej. Recepcionista → Profesor). SQL: sql/supabase_todo_reasignar.sql. Docs: docs/CONFIGURACION.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2267,7 +2359,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2714,9 +2806,20 @@
         <v>Modal Detalle (Concepto y Beneficiario): clic en cualquier importe abre modal Movimientos con las filas que lo componen (sucursal, moneda/TC, exclusión Saldo Inicial; G/P con egresos negativos), total al pie y export Excel. Carga base_everfit suma detalle, medio y observaciones. everfit-release.json v1.38.</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>1.39</v>
+      </c>
+      <c r="B41" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Dashboard: filtro Período (default último año; años; todo el histórico) aplicado a tarjetas, gráfico, Flujo, ratios, Detalle, Movimientos y PDF; Proy. solo si incluye el mes en curso. Gráfico G/P con tendencia y variación vs mes anterior. Botón PDF con filtros activos resaltados, importes en miles y sin meses proyectados. everfit-release.json v1.39.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.40: mes en curso fuera de totales, orden de columnas Total/Proy. y alertas de desvío
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E104"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2144,16 +2144,50 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B103" t="str">
+        <v>17:00</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Flujo por mes – mes en curso, orden de columnas y alertas (criterio Fornitalia)</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Mes en curso en celeste en tabla, ratios, gráfico (G/P en millones) y PDF, fuera de tarjetas, Total, ratios totales, variación y tendencia. Orden de columnas: meses → Total (solo cerrados) → Proy. Alertas de desvío vs mes anterior por concepto (ingresos) / beneficiario (egresos) con triángulo en el encabezado del mes y modal; umbral configurable en el modal Proyección (config_dashboard.alerta_desvio_pct, sql/supabase_config_dashboard_alerta_desvio.sql aplicado). Docs: DASHBOARD.md, PROYECCION_FLUJO.md.</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B104" t="str">
+        <v>17:05</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Despliegue v1.40</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Mes en curso en celeste fuera de totales, orden de columnas meses → Total → Proy. y alertas de desvío vs mes anterior; everfit-release.json v1.40. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E102"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E104"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -2257,39 +2291,55 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Dashboard – reporte PDF</v>
+        <v>Flujo por mes – mes en curso y orden de columnas</v>
       </c>
       <c r="B13" t="str">
-        <v>Botón PDF en la barra de filtros: reporte imprimible (Guardar como PDF) con filtros activos resaltados, importes en miles, tarjetas, gráfico G/P y tabla Flujo por mes + ratios del período elegido, sin meses proyectados. Docs: docs/DASHBOARD.md.</v>
+        <v>El mes en curso se ve en celeste (tabla, ratios, gráfico con G/P en millones y PDF) pero no suma en tarjetas, Total, ratios totales, variación ni tendencia. Columnas: meses → Total (solo meses cerrados) → Proy. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Detalle por Concepto / Beneficiario – movimientos</v>
+        <v>Flujo por mes – alertas de desvío</v>
       </c>
       <c r="B14" t="str">
-        <v>En el modal Detalle (clic en fila del Flujo por mes), cualquier importe de ambas solapas abre el listado de movimientos que lo componen: fecha de pago, tipo, concepto, beneficiario, centro de costos, detalle, medio, sucursal, real/pendiente, observaciones e importe, con total al pie y export Excel. Respeta sucursal, moneda ARS/USD y exclusión Saldo Inicial. Docs: docs/DASHBOARD.md.</v>
+        <v>Triángulo en el encabezado del mes cuando un concepto de ingreso o beneficiario de egreso varía más del umbral % vs el mes anterior; modal con el detalle (verde favorable / rojo desfavorable). Umbral por usuario en el modal Proyección (config_dashboard.alerta_desvio_pct). Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Sedes – catálogo ABM</v>
+        <v>Dashboard – reporte PDF</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+        <v>Botón PDF en la barra de filtros: reporte imprimible (Guardar como PDF) con filtros activos resaltados, importes en miles, tarjetas, gráfico G/P y tabla Flujo por mes + ratios del período elegido, sin meses proyectados. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>Detalle por Concepto / Beneficiario – movimientos</v>
+      </c>
+      <c r="B16" t="str">
+        <v>En el modal Detalle (clic en fila del Flujo por mes), cualquier importe de ambas solapas abre el listado de movimientos que lo componen: fecha de pago, tipo, concepto, beneficiario, centro de costos, detalle, medio, sucursal, real/pendiente, observaciones e importe, con total al pie y export Excel. Respeta sucursal, moneda ARS/USD y exclusión Saldo Inicial. Docs: docs/DASHBOARD.md.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Sedes – catálogo ABM</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>Configuración – reasignar To-Do</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B18" t="str">
         <v>Menú Configuración (permiso ver_configuracion, default Admin/Encargado). Reasignar una, varias o todas las tareas abiertas de un usuario a otro, o de un perfil a otro (p. ej. Recepcionista → Profesor). SQL: sql/supabase_todo_reasignar.sql. Docs: docs/CONFIGURACION.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2359,7 +2409,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2817,9 +2867,20 @@
         <v>Dashboard: filtro Período (default último año; años; todo el histórico) aplicado a tarjetas, gráfico, Flujo, ratios, Detalle, Movimientos y PDF; Proy. solo si incluye el mes en curso. Gráfico G/P con tendencia y variación vs mes anterior. Botón PDF con filtros activos resaltados, importes en miles y sin meses proyectados. everfit-release.json v1.39.</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>1.40</v>
+      </c>
+      <c r="B42" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Flujo por mes con criterio Fornitalia: mes en curso en celeste (tabla, ratios, gráfico con G/P en millones y PDF) fuera de tarjetas, Total, ratios totales, variación y tendencia; orden de columnas meses → Total (solo cerrados) → Proy.; alertas de desvío vs mes anterior por concepto (ingresos) / beneficiario (egresos) con modal y umbral por usuario en el modal Proyección (config_dashboard.alerta_desvio_pct). everfit-release.json v1.40.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.41: histórico al último mes cerrado en las tarjetas
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E104"/>
+  <dimension ref="A1:E106"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2178,16 +2178,50 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B105" t="str">
+        <v>08:27</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Tarjetas – valor histórico al último mes cerrado</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Si el Período no es Todo el histórico, debajo de Total ingresos, Total egresos y G/P Total se muestra en letra más chica «Histórico al dd/mm/aaaa» (último día del último mes cerrado, Argentina) con el acumulado de todos los meses cerrados, respetando sucursal y moneda. También en las tarjetas del PDF. Docs: DASHBOARD.md.</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B106" t="str">
+        <v>08:27</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Despliegue v1.41</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Histórico al último mes cerrado en las tarjetas del Dashboard y del PDF; everfit-release.json v1.41. Push a main y vercel --prod.</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E104"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E106"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -2291,55 +2325,63 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Flujo por mes – mes en curso y orden de columnas</v>
+        <v>Tarjetas – histórico al último mes cerrado</v>
       </c>
       <c r="B13" t="str">
-        <v>El mes en curso se ve en celeste (tabla, ratios, gráfico con G/P en millones y PDF) pero no suma en tarjetas, Total, ratios totales, variación ni tendencia. Columnas: meses → Total (solo meses cerrados) → Proy. Docs: docs/DASHBOARD.md.</v>
+        <v>Con un Período distinto de Todo el histórico, cada tarjeta (ingresos, egresos, G/P) muestra debajo el acumulado histórico de los meses cerrados con el título «Histórico al dd/mm/aaaa». Incluido en el PDF. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Flujo por mes – alertas de desvío</v>
+        <v>Flujo por mes – mes en curso y orden de columnas</v>
       </c>
       <c r="B14" t="str">
-        <v>Triángulo en el encabezado del mes cuando un concepto de ingreso o beneficiario de egreso varía más del umbral % vs el mes anterior; modal con el detalle (verde favorable / rojo desfavorable). Umbral por usuario en el modal Proyección (config_dashboard.alerta_desvio_pct). Docs: docs/DASHBOARD.md.</v>
+        <v>El mes en curso se ve en celeste (tabla, ratios, gráfico con G/P en millones y PDF) pero no suma en tarjetas, Total, ratios totales, variación ni tendencia. Columnas: meses → Total (solo meses cerrados) → Proy. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Dashboard – reporte PDF</v>
+        <v>Flujo por mes – alertas de desvío</v>
       </c>
       <c r="B15" t="str">
-        <v>Botón PDF en la barra de filtros: reporte imprimible (Guardar como PDF) con filtros activos resaltados, importes en miles, tarjetas, gráfico G/P y tabla Flujo por mes + ratios del período elegido, sin meses proyectados. Docs: docs/DASHBOARD.md.</v>
+        <v>Triángulo en el encabezado del mes cuando un concepto de ingreso o beneficiario de egreso varía más del umbral % vs el mes anterior; modal con el detalle (verde favorable / rojo desfavorable). Umbral por usuario en el modal Proyección (config_dashboard.alerta_desvio_pct). Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Detalle por Concepto / Beneficiario – movimientos</v>
+        <v>Dashboard – reporte PDF</v>
       </c>
       <c r="B16" t="str">
-        <v>En el modal Detalle (clic en fila del Flujo por mes), cualquier importe de ambas solapas abre el listado de movimientos que lo componen: fecha de pago, tipo, concepto, beneficiario, centro de costos, detalle, medio, sucursal, real/pendiente, observaciones e importe, con total al pie y export Excel. Respeta sucursal, moneda ARS/USD y exclusión Saldo Inicial. Docs: docs/DASHBOARD.md.</v>
+        <v>Botón PDF en la barra de filtros: reporte imprimible (Guardar como PDF) con filtros activos resaltados, importes en miles, tarjetas, gráfico G/P y tabla Flujo por mes + ratios del período elegido, sin meses proyectados. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Sedes – catálogo ABM</v>
+        <v>Detalle por Concepto / Beneficiario – movimientos</v>
       </c>
       <c r="B17" t="str">
-        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+        <v>En el modal Detalle (clic en fila del Flujo por mes), cualquier importe de ambas solapas abre el listado de movimientos que lo componen: fecha de pago, tipo, concepto, beneficiario, centro de costos, detalle, medio, sucursal, real/pendiente, observaciones e importe, con total al pie y export Excel. Respeta sucursal, moneda ARS/USD y exclusión Saldo Inicial. Docs: docs/DASHBOARD.md.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>Sedes – catálogo ABM</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Menú Sedes (Admin): alta/edición/activar-desactivar. Alimenta asignación de sedes en Seguridad y opciones de sede del To-Do. SQL: sql/supabase_sedes.sql. Docs: docs/SEDES.md.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>Configuración – reasignar To-Do</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B19" t="str">
         <v>Menú Configuración (permiso ver_configuracion, default Admin/Encargado). Reasignar una, varias o todas las tareas abiertas de un usuario a otro, o de un perfil a otro (p. ej. Recepcionista → Profesor). SQL: sql/supabase_todo_reasignar.sql. Docs: docs/CONFIGURACION.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2409,7 +2451,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2878,9 +2920,20 @@
         <v>Flujo por mes con criterio Fornitalia: mes en curso en celeste (tabla, ratios, gráfico con G/P en millones y PDF) fuera de tarjetas, Total, ratios totales, variación y tendencia; orden de columnas meses → Total (solo cerrados) → Proy.; alertas de desvío vs mes anterior por concepto (ingresos) / beneficiario (egresos) con modal y umbral por usuario en el modal Proyección (config_dashboard.alerta_desvio_pct). everfit-release.json v1.40.</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>1.41</v>
+      </c>
+      <c r="B43" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Tarjetas del Dashboard: si el Período no es Todo el histórico, debajo de cada valor se muestra «Histórico al dd/mm/aaaa» (último día del último mes cerrado) con el acumulado de todos los meses cerrados, respetando sucursal y moneda; también en el PDF. everfit-release.json v1.41.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>